<commit_message>
Commiting close to production version
</commit_message>
<xml_diff>
--- a/Simulation_studies/cir_parameter_comparison_Xdim1.xlsx
+++ b/Simulation_studies/cir_parameter_comparison_Xdim1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,10 +446,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Log_like</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Abs Error</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Rel Error (%)</t>
         </is>
@@ -462,16 +472,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7263904006370904</v>
+        <v>0.4919758308668359</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7810834903898229</v>
+        <v>0.5128314427850377</v>
       </c>
       <c r="D2" t="n">
-        <v>0.05469308975273257</v>
+        <v>0.001081575510092363</v>
       </c>
       <c r="E2" t="n">
-        <v>7.002207885028572</v>
+        <v>28241.50550381297</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.02085561191820173</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.066757647491542</v>
       </c>
     </row>
     <row r="3">
@@ -481,16 +497,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2038190635832954</v>
+        <v>0.2458204014020154</v>
       </c>
       <c r="C3" t="n">
-        <v>0.206662525762542</v>
+        <v>0.2454983203324685</v>
       </c>
       <c r="D3" t="n">
-        <v>0.002843462179246636</v>
+        <v>0.0002121600974180942</v>
       </c>
       <c r="E3" t="n">
-        <v>1.375896364739978</v>
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0003220810695468423</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.1311948159607206</v>
       </c>
     </row>
     <row r="4">
@@ -500,16 +522,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.432963965159729</v>
+        <v>0.1016773282354888</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4434765472062681</v>
+        <v>0.1027856128487651</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01051258204653904</v>
+        <v>0.002083985722729393</v>
       </c>
       <c r="E4" t="n">
-        <v>2.370493346889317</v>
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.001108284613276334</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.078248776807919</v>
       </c>
     </row>
     <row r="5">
@@ -519,16 +547,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.1864222645217601</v>
+        <v>-0.2950667018054884</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.03076030927590256</v>
+        <v>-0.2875444412891958</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1556619552458575</v>
+        <v>0.08257822516148805</v>
       </c>
       <c r="E5" t="n">
-        <v>-506.0480824482545</v>
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.007522260516292678</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-2.616034058097899</v>
       </c>
     </row>
     <row r="6">
@@ -538,16 +572,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0004332388415225674</v>
+        <v>0.0005763261994719503</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0003723418220274678</v>
+        <v>0.0005758831230580474</v>
       </c>
       <c r="D6" t="n">
-        <v>6.089701949509957e-05</v>
+        <v>6.640387339229753e-06</v>
       </c>
       <c r="E6" t="n">
-        <v>16.35513818015511</v>
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.430764139029108e-07</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.07693860024063423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commiting close to final versions of all
</commit_message>
<xml_diff>
--- a/Simulation_studies/cir_parameter_comparison_Xdim1.xlsx
+++ b/Simulation_studies/cir_parameter_comparison_Xdim1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25ec18ff9d9d96f3/KU^J MAT-OEK/Kandidat/Thesis/Thesis_linear_CDS/Simulation_studies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_085D48DF5662143F6759B85657245E3FB48F88CD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A87D490C-7D9B-4CE5-BCC6-A92929F32241}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_085D63071368DCDFEF657C954B245E3FB48F88C6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{239D23CD-9F83-40C2-9695-CE22982980BF}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -112,8 +112,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -426,7 +432,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -435,7 +441,7 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -450,22 +456,22 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0.95320249429003379</v>
+        <v>0.91993941467613261</v>
       </c>
       <c r="C2">
         <v>1.072839344173294</v>
       </c>
       <c r="D2">
-        <v>2.3870654240594522E-2</v>
+        <v>2.6230116291705269E-2</v>
       </c>
       <c r="E2">
-        <v>18176.981343078271</v>
+        <v>10799.501986751289</v>
       </c>
       <c r="F2">
-        <v>0.1196368498832602</v>
+        <v>0.15289992949716141</v>
       </c>
       <c r="G2">
-        <v>11.151422674142291</v>
+        <v>14.251894314612651</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -473,22 +479,22 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>0.96266261476040038</v>
+        <v>0.99981756306718983</v>
       </c>
       <c r="C3">
         <v>0.91711405366737031</v>
       </c>
       <c r="D3">
-        <v>1.8805970577953801E-2</v>
+        <v>2.2831906002530909E-2</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>4.5548561093030071E-2</v>
+        <v>8.2703509399819519E-2</v>
       </c>
       <c r="G3">
-        <v>4.9665099897760543</v>
+        <v>9.0177998111688957</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -496,22 +502,22 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>1.0665317626733011</v>
+        <v>1.1135429387882041</v>
       </c>
       <c r="C4">
         <v>1.0565655119030479</v>
       </c>
       <c r="D4">
-        <v>1.841254925748205E-2</v>
+        <v>1.9724667831507621E-2</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>9.9662507702529268E-3</v>
+        <v>5.6977426885155953E-2</v>
       </c>
       <c r="G4">
-        <v>0.94326860549347968</v>
+        <v>5.3927017532997299</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -519,22 +525,22 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>-0.84224179019178091</v>
+        <v>-0.39875914188481038</v>
       </c>
       <c r="C5">
-        <v>-0.53689030720838971</v>
+        <v>-0.22625752114002429</v>
       </c>
       <c r="D5">
-        <v>0.48049692608532241</v>
+        <v>0.46734668517420058</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0.30535148298339121</v>
+        <v>0.17250162074478601</v>
       </c>
       <c r="G5">
-        <v>-56.874091203302633</v>
+        <v>-76.241275815105254</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -542,22 +548,22 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>3.9833802882099046E-3</v>
+        <v>1.9451700114322661E-2</v>
       </c>
       <c r="C6">
         <v>2.8955489524110648E-4</v>
       </c>
       <c r="D6">
-        <v>2.6461780681967581E-5</v>
+        <v>1.3439310959254119E-4</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>3.6938253929687981E-3</v>
+        <v>1.916214521908155E-2</v>
       </c>
       <c r="G6">
-        <v>1275.690880616273</v>
+        <v>6617.7935631603177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>